<commit_message>
fix(formats): harden container and image readers
</commit_message>
<xml_diff>
--- a/tests/fixtures/formats/displayed.xlsx
+++ b/tests/fixtures/formats/displayed.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="urn:r">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="Summary" r:id="sheet"/>
   </sheets>
@@ -8,22 +8,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
     <row r="1">
       <c r="A1">
-        <v>Formula</v>
-      </c>
-      <c r="B1">
-        <v>Displayed</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
         <f>SUM(1,2)</f>
-        <v>3</v>
-      </c>
-      <c r="B2">
         <v>3</v>
       </c>
     </row>

</xml_diff>